<commit_message>
OpenGrid MVP: AI-assisted geospatial data retrieval system
Includes: AI planning agent, multi-provider geocoding (AMap/Baidu/Nominatim), 9 data source clients, GeoJSON output pipeline, test suite, and documentation
</commit_message>
<xml_diff>
--- a/opengridworks.xlsx
+++ b/opengridworks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\实习\WRI\5.AI数据集\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D753BB2B-2F3E-40BB-814B-2A8F50CD84A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CF19BB-EC71-4E0B-8272-4144AB5A50AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="116">
   <si>
     <t>Source</t>
   </si>
@@ -36,30 +36,15 @@
     <t>License</t>
   </si>
   <si>
-    <t>EIA</t>
-  </si>
-  <si>
-    <t>Power plant attributes and capacity (EIA-860M). Source: U.S. Energy Information Administration.</t>
-  </si>
-  <si>
     <t>Basemap tiles and geospatial reference layers</t>
   </si>
   <si>
-    <t>HIFLD</t>
-  </si>
-  <si>
     <t>Transmission lines, substations, and natural gas pipeline geometry</t>
   </si>
   <si>
-    <t>FRA / BTS NARN</t>
-  </si>
-  <si>
     <t>North American Rail Network linework (rail right-of-way overlays)</t>
   </si>
   <si>
-    <t>FHWA / BTS NHS</t>
-  </si>
-  <si>
     <t>National Highway System centerlines (interstates and principal arterials)</t>
   </si>
   <si>
@@ -69,9 +54,6 @@
     <t>West-wide designated federal energy corridors</t>
   </si>
   <si>
-    <t>USACE NWN</t>
-  </si>
-  <si>
     <t>National Waterway Network (navigable commercial waterways)</t>
   </si>
   <si>
@@ -84,9 +66,6 @@
     <t>WRI Aqueduct 4.0</t>
   </si>
   <si>
-    <t>Power infrastructure geometries (substations, transmission lines, generation assets) via the OpenStreetMap power layer</t>
-  </si>
-  <si>
     <t>ODbL 1.0</t>
   </si>
   <si>
@@ -97,9 +76,6 @@
   </si>
   <si>
     <t>OurGridFuture</t>
-  </si>
-  <si>
-    <t>AFDC / DOE</t>
   </si>
   <si>
     <t>EV charging station locations via the Alternative Fuels Data Center</t>
@@ -316,9 +292,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>https://www.geofabrik.de/data/</t>
-  </si>
-  <si>
     <t>涵盖变电站、各级输电线路、分布式发电资产矢量几何数据集</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -369,10 +342,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>https://ngda-transportation-geoplatform.hub.arcgis.com/api/search/v1/collections/dataset/items/06037f2b23ff401aa1d379c2632a58f6</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>未来大规模石油输送管线、天然气及氢气管道网络，以及超高压输电与配电基础设施选址的优先优化区域</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -647,6 +616,153 @@
   </si>
   <si>
     <t>国家公路系统</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>AFDC / DOE</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>FRA / BTS NARN</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>FHWA / BTS NHS</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>HIFLD</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://services7.arcgis.com/n1YM8pTrFmm7L4hs/ArcGIS/rest/services/Waterway_Networks/FeatureServer/1</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>USACE NWN</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>EIA</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Power plant attributes and capacity (EIA-860M). Source: U.S. Energy Information Administration.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.geofabrik.de/data/</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Power infrastructure geometries (substations, transmission lines, generation assets) via the OpenStreetMap power layer</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>key</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>0qNhEM4COsSscqaKG5N4UskMtfKGPctWZvhsAsqk</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>4tre2lnAZyeb6LbYlw0PR1t4WFOGFqpPlhd4RMFH</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t>是否可以选择时间</t>
+    </r>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>支持：YEAR</t>
+  </si>
+  <si>
+    <t>支持：YEAR</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>NAN</t>
+  </si>
+  <si>
+    <t>支持：SOURCEDATE</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>支持：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>DATE_MOD</t>
+    </r>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>支持：period / start / end</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>NASA / USGS</t>
+  </si>
+  <si>
+    <t>MODIS Land Cover Type (MCD12Q1)</t>
+  </si>
+  <si>
+    <t>土地利用与覆盖</t>
+  </si>
+  <si>
+    <t>全球年度土地覆盖产品，基于IGBP分类系统，提供500米分辨率的地表覆盖类型数据。</t>
+  </si>
+  <si>
+    <t>U.S. Government Works; public domain</t>
+  </si>
+  <si>
+    <t>MODIS/061/MCD12Q1</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://search.earthdata.nasa.gov/search/granules?p=C2484079608-LPCLOUD&amp;q=MCD12Q1</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Raster (GEE)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t>可用性</t>
+    </r>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>全球</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>美国</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -654,7 +770,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -721,8 +837,36 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="等线"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -732,6 +876,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -749,24 +917,92 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1048,462 +1284,610 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="13.9"/>
   <cols>
-    <col min="1" max="1" width="20.265625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="51.53125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="20" style="3" customWidth="1"/>
-    <col min="4" max="4" width="20.265625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="31.53125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="36.86328125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="17.265625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="45.53125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="20.265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="51.53125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.265625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31.53125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="36.86328125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="45.53125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14.796875" customWidth="1"/>
+    <col min="11" max="11" width="18.265625" style="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:11" ht="27.75">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K1" s="31" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="4" customFormat="1" ht="41.65">
+      <c r="A2" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="K2" s="32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" s="4" customFormat="1" ht="70.900000000000006">
+      <c r="A3" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="K3" s="32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="30" customFormat="1" ht="41.65">
+      <c r="A4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" s="32" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" s="9" customFormat="1" ht="69.400000000000006">
+      <c r="A5" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="K5" s="32" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" s="7" customFormat="1" ht="97.15">
+      <c r="A6" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="F6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="K6" s="32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" s="7" customFormat="1" ht="41.65">
+      <c r="A7" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="K7" s="32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" s="7" customFormat="1" ht="69.400000000000006">
+      <c r="A8" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="G8" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>2</v>
+      <c r="H8" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="J8" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="K8" s="32" t="s">
+        <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="41.65">
-      <c r="A2" s="5" t="s">
+    <row r="9" spans="1:11" s="7" customFormat="1" ht="69.400000000000006">
+      <c r="A9" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="K9" s="32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="41.65">
+      <c r="A10" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="C10" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
+      <c r="D10" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="I10" s="22"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="32" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="41.65">
+      <c r="A11" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="83.25">
+      <c r="A12" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="32" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="69.400000000000006">
+      <c r="A13" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="22" t="s">
         <v>30</v>
       </c>
+      <c r="C13" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="H13" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="32" t="s">
+        <v>115</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" ht="41.65">
-      <c r="A3" s="4" t="s">
+    <row r="14" spans="1:11" ht="55.5">
+      <c r="A14" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="32" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" s="3" customFormat="1" ht="55.5">
+      <c r="A15" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C15" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>28</v>
+      <c r="G15" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="32" t="s">
+        <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="41.65">
-      <c r="A4" s="4" t="s">
+    <row r="16" spans="1:11" s="3" customFormat="1" ht="111">
+      <c r="A16" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>27</v>
+      <c r="C16" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="32" t="s">
+        <v>114</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="111">
-      <c r="A5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5" s="4" t="s">
+    <row r="17" spans="1:10" ht="41.65">
+      <c r="A17" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="83.25">
-      <c r="A6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="97.15">
-      <c r="A7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="41.65">
-      <c r="A8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="70.900000000000006">
-      <c r="A9" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="83.25">
-      <c r="A10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="97.15">
-      <c r="A11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="41.65">
-      <c r="A12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="69.400000000000006">
-      <c r="A13" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="55.5">
-      <c r="A14" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" s="6" customFormat="1" ht="55.5">
-      <c r="A15" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" s="6" customFormat="1" ht="111">
-      <c r="A16" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H17">
-    <sortCondition ref="C1:C17"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H18">
+    <sortCondition ref="C1:C18"/>
   </sortState>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="H9" r:id="rId1" display="https://www.usa.gov/government-works" xr:uid="{7ED09C60-6D48-47B3-A37E-1DB64DAFB871}"/>
-    <hyperlink ref="H11" r:id="rId2" display="https://www.usa.gov/government-works" xr:uid="{15664D0A-0A0D-4330-B7B1-E3EA0388B1BA}"/>
-    <hyperlink ref="H7" r:id="rId3" display="https://www.usa.gov/government-works" xr:uid="{8CBD223E-6947-4805-B5EB-1846B4D1CB6D}"/>
-    <hyperlink ref="H6" r:id="rId4" display="https://www.usa.gov/government-works" xr:uid="{6FE46663-19E5-4303-9C9C-3D0306C4FBF9}"/>
-    <hyperlink ref="H8" r:id="rId5" display="https://www.usa.gov/government-works" xr:uid="{0B1ABCF4-66C5-4D8E-BFF5-F442830327F5}"/>
-    <hyperlink ref="H5" r:id="rId6" display="https://www.usa.gov/government-works" xr:uid="{A47F53A1-4D7D-4F40-9D09-0298B5C0B491}"/>
+    <hyperlink ref="H3" r:id="rId1" display="https://www.usa.gov/government-works" xr:uid="{7ED09C60-6D48-47B3-A37E-1DB64DAFB871}"/>
+    <hyperlink ref="H6" r:id="rId2" display="https://www.usa.gov/government-works" xr:uid="{15664D0A-0A0D-4330-B7B1-E3EA0388B1BA}"/>
+    <hyperlink ref="H9" r:id="rId3" display="https://www.usa.gov/government-works" xr:uid="{8CBD223E-6947-4805-B5EB-1846B4D1CB6D}"/>
+    <hyperlink ref="H8" r:id="rId4" display="https://www.usa.gov/government-works" xr:uid="{6FE46663-19E5-4303-9C9C-3D0306C4FBF9}"/>
+    <hyperlink ref="H11" r:id="rId5" display="https://www.usa.gov/government-works" xr:uid="{0B1ABCF4-66C5-4D8E-BFF5-F442830327F5}"/>
+    <hyperlink ref="H7" r:id="rId6" display="https://www.usa.gov/government-works" xr:uid="{A47F53A1-4D7D-4F40-9D09-0298B5C0B491}"/>
     <hyperlink ref="B14" r:id="rId7" display="https://doi.org/10.57931/2550666" xr:uid="{8374E5FA-616E-464A-BD7D-E5A84775D8F4}"/>
     <hyperlink ref="H15" r:id="rId8" display="https://creativecommons.org/licenses/by/4.0/" xr:uid="{84FB93B8-233D-41CE-85A3-E21A1DC00D78}"/>
-    <hyperlink ref="B16" r:id="rId9" display="https://doi.org/10.46830/writn.23.00061" xr:uid="{D6F5ED5C-0D8B-4778-A799-ED2B2A19077F}"/>
-    <hyperlink ref="H16" r:id="rId10" display="https://creativecommons.org/licenses/by/4.0/legalcode" xr:uid="{49084FCF-BFF6-4811-B636-B5AB5FF9E580}"/>
-    <hyperlink ref="A12" r:id="rId11" display="https://www.openstreetmap.org/copyright" xr:uid="{68339B7F-624B-42B3-9FA3-A7D87738261C}"/>
-    <hyperlink ref="H12" r:id="rId12" display="https://opendatacommons.org/licenses/odbl/1.0/" xr:uid="{F46884D5-FD0A-42BF-BA38-745C2E64FCE5}"/>
-    <hyperlink ref="H10" r:id="rId13" display="https://creativecommons.org/licenses/by/4.0/" xr:uid="{E5452CA7-2666-49DF-B763-A60B2800C673}"/>
-    <hyperlink ref="H13" r:id="rId14" display="https://ourgridfuture.org/" xr:uid="{C49FBD35-C3AA-4584-A9B4-6016C77AC0D3}"/>
-    <hyperlink ref="H3" r:id="rId15" display="https://www.usa.gov/government-works" xr:uid="{3928C090-5AB7-4AE8-973A-4CED66CA2D25}"/>
-    <hyperlink ref="B4" r:id="rId16" display="https://www.submarinecablemap.com/" xr:uid="{745C7DA8-91CE-4DC2-BDA6-D78C0B816A63}"/>
-    <hyperlink ref="H4" r:id="rId17" display="https://creativecommons.org/licenses/by-sa/4.0/" xr:uid="{29885042-96EB-40C6-8383-C9E31F3E7097}"/>
-    <hyperlink ref="D9" r:id="rId18" xr:uid="{4C4B5D5A-B022-46C5-8A1D-2D8E33E20ABD}"/>
-    <hyperlink ref="E9" r:id="rId19" xr:uid="{81106B1D-3C85-4C13-BEF7-62AEB5FAE7D6}"/>
-    <hyperlink ref="E11" r:id="rId20" xr:uid="{558D3C3A-E40C-442A-8B8C-6CCCE6DED592}"/>
-    <hyperlink ref="D11" r:id="rId21" xr:uid="{38710F5A-05D3-44F7-B940-CBB85684CD1C}"/>
-    <hyperlink ref="D13" r:id="rId22" xr:uid="{AC16D8BE-7BDC-47C4-A065-CE756312C112}"/>
-    <hyperlink ref="E12" r:id="rId23" xr:uid="{C9305481-B3F0-4094-A87D-4AAE1F505422}"/>
-    <hyperlink ref="D10" r:id="rId24" xr:uid="{EA415C13-2F21-4987-BCCA-480574A258E5}"/>
-    <hyperlink ref="E7" r:id="rId25" xr:uid="{D3C4E117-9A37-41B8-A3AC-5C7F1DD73064}"/>
-    <hyperlink ref="D6" r:id="rId26" xr:uid="{91CF1C71-DD1E-498F-9FA1-36EAA535612D}"/>
-    <hyperlink ref="D7" r:id="rId27" xr:uid="{06A6BF19-F19E-44BA-A96C-761F96C5E8B0}"/>
-    <hyperlink ref="E6" r:id="rId28" xr:uid="{FA002878-3638-4512-9CE1-21BEE31D7E31}"/>
-    <hyperlink ref="D5" r:id="rId29" xr:uid="{1379E54D-D43E-46B6-8FBA-C72B7074D686}"/>
-    <hyperlink ref="E5" r:id="rId30" xr:uid="{28C13DBF-092B-4BB6-84E1-11857F26FA60}"/>
-    <hyperlink ref="D8" r:id="rId31" xr:uid="{83A91E8D-FEAE-40A0-B50C-44D72DE3251A}"/>
-    <hyperlink ref="D14" r:id="rId32" xr:uid="{BB6E15F3-EC5D-484B-B3B1-94FE77BC8B33}"/>
-    <hyperlink ref="D3" r:id="rId33" xr:uid="{8D3F8D5C-C87B-44CC-9AB4-146CE51FFA19}"/>
-    <hyperlink ref="E3" r:id="rId34" xr:uid="{9E5DA780-3AEB-45B8-A88B-B7172F9B6D5F}"/>
-    <hyperlink ref="D4" r:id="rId35" xr:uid="{DC57DF95-5447-47E4-95A6-07547C144430}"/>
+    <hyperlink ref="A4" r:id="rId9" display="https://www.openstreetmap.org/copyright" xr:uid="{68339B7F-624B-42B3-9FA3-A7D87738261C}"/>
+    <hyperlink ref="H4" r:id="rId10" display="https://opendatacommons.org/licenses/odbl/1.0/" xr:uid="{F46884D5-FD0A-42BF-BA38-745C2E64FCE5}"/>
+    <hyperlink ref="H12" r:id="rId11" display="https://creativecommons.org/licenses/by/4.0/" xr:uid="{E5452CA7-2666-49DF-B763-A60B2800C673}"/>
+    <hyperlink ref="H13" r:id="rId12" display="https://ourgridfuture.org/" xr:uid="{C49FBD35-C3AA-4584-A9B4-6016C77AC0D3}"/>
+    <hyperlink ref="H2" r:id="rId13" display="https://www.usa.gov/government-works" xr:uid="{3928C090-5AB7-4AE8-973A-4CED66CA2D25}"/>
+    <hyperlink ref="B10" r:id="rId14" display="https://www.submarinecablemap.com/" xr:uid="{745C7DA8-91CE-4DC2-BDA6-D78C0B816A63}"/>
+    <hyperlink ref="H10" r:id="rId15" display="https://creativecommons.org/licenses/by-sa/4.0/" xr:uid="{29885042-96EB-40C6-8383-C9E31F3E7097}"/>
+    <hyperlink ref="D3" r:id="rId16" xr:uid="{4C4B5D5A-B022-46C5-8A1D-2D8E33E20ABD}"/>
+    <hyperlink ref="E3" r:id="rId17" xr:uid="{81106B1D-3C85-4C13-BEF7-62AEB5FAE7D6}"/>
+    <hyperlink ref="E6" r:id="rId18" xr:uid="{558D3C3A-E40C-442A-8B8C-6CCCE6DED592}"/>
+    <hyperlink ref="D6" r:id="rId19" xr:uid="{38710F5A-05D3-44F7-B940-CBB85684CD1C}"/>
+    <hyperlink ref="D13" r:id="rId20" xr:uid="{AC16D8BE-7BDC-47C4-A065-CE756312C112}"/>
+    <hyperlink ref="E4" r:id="rId21" xr:uid="{C9305481-B3F0-4094-A87D-4AAE1F505422}"/>
+    <hyperlink ref="D12" r:id="rId22" xr:uid="{EA415C13-2F21-4987-BCCA-480574A258E5}"/>
+    <hyperlink ref="E9" r:id="rId23" xr:uid="{D3C4E117-9A37-41B8-A3AC-5C7F1DD73064}"/>
+    <hyperlink ref="D8" r:id="rId24" xr:uid="{91CF1C71-DD1E-498F-9FA1-36EAA535612D}"/>
+    <hyperlink ref="D9" r:id="rId25" xr:uid="{06A6BF19-F19E-44BA-A96C-761F96C5E8B0}"/>
+    <hyperlink ref="E8" r:id="rId26" xr:uid="{FA002878-3638-4512-9CE1-21BEE31D7E31}"/>
+    <hyperlink ref="D7" r:id="rId27" xr:uid="{1379E54D-D43E-46B6-8FBA-C72B7074D686}"/>
+    <hyperlink ref="E7" r:id="rId28" xr:uid="{28C13DBF-092B-4BB6-84E1-11857F26FA60}"/>
+    <hyperlink ref="D11" r:id="rId29" xr:uid="{83A91E8D-FEAE-40A0-B50C-44D72DE3251A}"/>
+    <hyperlink ref="D14" r:id="rId30" xr:uid="{BB6E15F3-EC5D-484B-B3B1-94FE77BC8B33}"/>
+    <hyperlink ref="D2" r:id="rId31" xr:uid="{8D3F8D5C-C87B-44CC-9AB4-146CE51FFA19}"/>
+    <hyperlink ref="E2" r:id="rId32" xr:uid="{9E5DA780-3AEB-45B8-A88B-B7172F9B6D5F}"/>
+    <hyperlink ref="D10" r:id="rId33" xr:uid="{DC57DF95-5447-47E4-95A6-07547C144430}"/>
+    <hyperlink ref="D4" r:id="rId34" xr:uid="{767C79ED-F01D-4E67-BB58-D8A751A56F4C}"/>
+    <hyperlink ref="H16" r:id="rId35" display="https://creativecommons.org/licenses/by/4.0/legalcode" xr:uid="{49084FCF-BFF6-4811-B636-B5AB5FF9E580}"/>
+    <hyperlink ref="B16" r:id="rId36" display="https://doi.org/10.46830/writn.23.00061" xr:uid="{D6F5ED5C-0D8B-4778-A799-ED2B2A19077F}"/>
+    <hyperlink ref="D5" r:id="rId37" xr:uid="{F72B6806-4E0B-4939-B19F-0696B9059919}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="256" orientation="portrait" r:id="rId36"/>
+  <pageSetup paperSize="256" orientation="portrait" r:id="rId38"/>
 </worksheet>
 </file>
</xml_diff>